<commit_message>
final round of paper ficxes implemented. gemini ran on all abalations.
chore: update analysis outputs and gitignore for ablation studies

Updated binary Excel files across Hybrid, Prompt, and RAG ablation analyses with new statistical test results and bootstrap confidence intervals. Added consolidation and workstream reports to .gitignore
</commit_message>
<xml_diff>
--- a/Analysis/Hybrid_Ablation/hybrid_ablation_bootstrap_ci.xlsx
+++ b/Analysis/Hybrid_Ablation/hybrid_ablation_bootstrap_ci.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,7 +492,7 @@
         <v>0.8598290598290599</v>
       </c>
       <c r="E3" t="n">
-        <v>0.941880341880342</v>
+        <v>0.9452991452991452</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -619,10 +619,10 @@
         <v>0.1221709401709402</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1064784188034188</v>
+        <v>0.1068246794871795</v>
       </c>
       <c r="E8" t="n">
-        <v>0.138842094017094</v>
+        <v>0.138013782051282</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -645,10 +645,10 @@
         <v>0.04114529914529914</v>
       </c>
       <c r="D9" t="n">
-        <v>0.03655117521367521</v>
+        <v>0.03644871794871795</v>
       </c>
       <c r="E9" t="n">
-        <v>0.04615405982905983</v>
+        <v>0.04614102564102564</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -697,7 +697,7 @@
         <v>0.6410256410256411</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5521367521367522</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="E11" t="n">
         <v>0.7230769230769231</v>
@@ -711,7 +711,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -720,13 +720,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.9209621993127147</v>
+        <v>0.9213675213675213</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8831615120274913</v>
+        <v>0.8803418803418804</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9518900343642612</v>
+        <v>0.9555555555555556</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -763,7 +763,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -775,7 +775,7 @@
         <v>0.7692307692307693</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7076923076923077</v>
+        <v>0.7128205128205128</v>
       </c>
       <c r="E14" t="n">
         <v>0.8256410256410256</v>
@@ -789,7 +789,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.9432989690721649</v>
+        <v>0.9282051282051282</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9072164948453608</v>
+        <v>0.8923076923076924</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9742268041237113</v>
+        <v>0.9641025641025641</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -841,7 +841,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -853,10 +853,10 @@
         <v>0.1221709401709402</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1064784188034188</v>
+        <v>0.106632264957265</v>
       </c>
       <c r="E17" t="n">
-        <v>0.138842094017094</v>
+        <v>0.1381583333333333</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -876,13 +876,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.04632302405498281</v>
+        <v>0.04686324786324786</v>
       </c>
       <c r="D18" t="n">
-        <v>0.04038638316151202</v>
+        <v>0.04008974358974359</v>
       </c>
       <c r="E18" t="n">
-        <v>0.05281357388316151</v>
+        <v>0.05380769230769231</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -919,7 +919,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -931,7 +931,7 @@
         <v>0.6410256410256411</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5521367521367522</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="E20" t="n">
         <v>0.7230769230769231</v>
@@ -945,7 +945,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.8974358974358975</v>
+        <v>0.9209621993127147</v>
       </c>
       <c r="D21" t="n">
-        <v>0.8495726495726497</v>
+        <v>0.8831615120274915</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9384615384615385</v>
+        <v>0.9518900343642612</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.9128205128205128</v>
+        <v>0.9432989690721649</v>
       </c>
       <c r="D24" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.9072164948453608</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9487179487179487</v>
+        <v>0.9742268041237113</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1087,10 +1087,10 @@
         <v>0.1221709401709402</v>
       </c>
       <c r="D26" t="n">
-        <v>0.1064784188034188</v>
+        <v>0.107033547008547</v>
       </c>
       <c r="E26" t="n">
-        <v>0.138842094017094</v>
+        <v>0.1382825854700855</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1110,13 +1110,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.06588034188034189</v>
+        <v>0.04632302405498281</v>
       </c>
       <c r="D27" t="n">
-        <v>0.05507692307692307</v>
+        <v>0.04023625429553265</v>
       </c>
       <c r="E27" t="n">
-        <v>0.07743611111111112</v>
+        <v>0.05289959192439862</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>qwen</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1145,6 +1145,240 @@
         <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>default_params</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.6410256410256411</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.7230769230769231</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>kendall_tau</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.8974358974358975</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.8495726495726497</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.9384615384615385</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>kendall_tau</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>true_params</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>kendall_tau</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>default_params</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.7076923076923077</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.8256410256410256</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>top1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.9128205128205128</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>top1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>true_params</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>top1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>default_params</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0.1221709401709402</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.1063885683760684</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.1380770299145299</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0.06588034188034189</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.05536752136752137</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.07733771367521368</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>qwen</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>true_params</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>mae</t>
         </is>

</xml_diff>

<commit_message>
remoived true_params arm from hybrid ablation and paper changes
</commit_message>
<xml_diff>
--- a/Analysis/Hybrid_Ablation/hybrid_ablation_bootstrap_ci.xlsx
+++ b/Analysis/Hybrid_Ablation/hybrid_ablation_bootstrap_ci.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,21 +508,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0.7076923076923077</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0.8256410256410256</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>kendall_tau</t>
+          <t>top1</t>
         </is>
       </c>
     </row>
@@ -534,17 +534,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>default_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.9128205128205128</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7076923076923077</v>
+        <v>0.8717948717948718</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8256410256410256</v>
+        <v>0.9487179487179487</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -560,21 +560,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>extracted</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9128205128205128</v>
+        <v>0.1223461538461538</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.106991452991453</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9487179487179487</v>
+        <v>0.1382181623931624</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>top1</t>
+          <t>mae</t>
         </is>
       </c>
     </row>
@@ -586,28 +586,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0.04013247863247862</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0.03550844017094017</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0.04500010683760685</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>top1</t>
+          <t>mae</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -616,24 +616,24 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1221709401709402</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1068246794871795</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="E8" t="n">
-        <v>0.138013782051282</v>
+        <v>0.7230769230769231</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>mae</t>
+          <t>kendall_tau</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -642,43 +642,43 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.04114529914529914</v>
+        <v>0.9213675213675213</v>
       </c>
       <c r="D9" t="n">
-        <v>0.03644871794871795</v>
+        <v>0.8803418803418804</v>
       </c>
       <c r="E9" t="n">
-        <v>0.04614102564102564</v>
+        <v>0.9555555555555556</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>mae</t>
+          <t>kendall_tau</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>gemini</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.7128205128205128</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>0.8256410256410256</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>mae</t>
+          <t>top1</t>
         </is>
       </c>
     </row>
@@ -690,21 +690,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>default_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.9282051282051282</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.8923076923076924</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7230769230769231</v>
+        <v>0.9641025641025641</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>kendall_tau</t>
+          <t>top1</t>
         </is>
       </c>
     </row>
@@ -716,21 +716,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>extracted</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.9213675213675213</v>
+        <v>0.1223461538461538</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8803418803418804</v>
+        <v>0.1068290598290599</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9555555555555556</v>
+        <v>0.1382566239316239</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>kendall_tau</t>
+          <t>mae</t>
         </is>
       </c>
     </row>
@@ -742,28 +742,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0.04703846153846153</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0.04028621794871794</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0.05385940170940171</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>kendall_tau</t>
+          <t>mae</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -772,24 +772,24 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7128205128205128</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="E14" t="n">
-        <v>0.8256410256410256</v>
+        <v>0.7230769230769231</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>top1</t>
+          <t>kendall_tau</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -798,39 +798,39 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.9282051282051282</v>
+        <v>0.9209621993127147</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8923076923076924</v>
+        <v>0.8831615120274915</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9641025641025641</v>
+        <v>0.9518900343642612</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>top1</t>
+          <t>kendall_tau</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0.7076923076923077</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0.8256410256410256</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -841,48 +841,48 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>default_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.1221709401709402</v>
+        <v>0.9432989690721649</v>
       </c>
       <c r="D17" t="n">
-        <v>0.106632264957265</v>
+        <v>0.9072164948453608</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1381583333333333</v>
+        <v>0.9742268041237113</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>mae</t>
+          <t>top1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>extracted</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.04686324786324786</v>
+        <v>0.1223461538461538</v>
       </c>
       <c r="D18" t="n">
-        <v>0.04008974358974359</v>
+        <v>0.1073416666666667</v>
       </c>
       <c r="E18" t="n">
-        <v>0.05380769230769231</v>
+        <v>0.1384918803418803</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -893,22 +893,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gemini</t>
+          <t>gptoss</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.04649914089347079</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>0.04028339776632302</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>0.05321746134020618</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -945,7 +945,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.9209621993127147</v>
+        <v>0.8974358974358975</v>
       </c>
       <c r="D21" t="n">
-        <v>0.8831615120274915</v>
+        <v>0.8495726495726497</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9518900343642612</v>
+        <v>0.9384615384615385</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -971,48 +971,48 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>0.7076923076923077</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>0.8256410256410256</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>kendall_tau</t>
+          <t>top1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>default_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.9128205128205128</v>
       </c>
       <c r="D23" t="n">
-        <v>0.7076923076923077</v>
+        <v>0.8717948717948718</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8256410256410256</v>
+        <v>0.9487179487179487</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1023,362 +1023,50 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>extracted</t>
+          <t>default_params</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.9432989690721649</v>
+        <v>0.1223461538461538</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9072164948453608</v>
+        <v>0.1065852564102564</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9742268041237113</v>
+        <v>0.1382867521367522</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>top1</t>
+          <t>mae</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gptoss</t>
+          <t>qwen</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>true_params</t>
+          <t>extracted</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0.06605555555555556</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>0.05561068376068376</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0.07737179487179487</v>
       </c>
       <c r="F25" t="inlineStr">
-        <is>
-          <t>top1</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>default_params</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0.1221709401709402</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.107033547008547</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.1382825854700855</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>mae</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>extracted</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0.04632302405498281</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.04023625429553265</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0.05289959192439862</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>mae</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>gptoss</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>true_params</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>mae</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>default_params</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>0.6410256410256411</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0.7230769230769231</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>kendall_tau</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>extracted</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0.8974358974358975</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0.8495726495726497</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0.9384615384615385</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>kendall_tau</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>true_params</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>kendall_tau</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>default_params</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>0.7692307692307693</v>
-      </c>
-      <c r="D32" t="n">
-        <v>0.7076923076923077</v>
-      </c>
-      <c r="E32" t="n">
-        <v>0.8256410256410256</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>top1</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>extracted</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>0.9128205128205128</v>
-      </c>
-      <c r="D33" t="n">
-        <v>0.8717948717948718</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0.9487179487179487</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>top1</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>true_params</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>top1</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>default_params</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>0.1221709401709402</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0.1063885683760684</v>
-      </c>
-      <c r="E35" t="n">
-        <v>0.1380770299145299</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>mae</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>extracted</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>0.06588034188034189</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0.05536752136752137</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0.07733771367521368</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>mae</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>true_params</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="inlineStr">
         <is>
           <t>mae</t>
         </is>

</xml_diff>